<commit_message>
feat(calculators): adding support for custom inputs for 4.4.1.1 method 2
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/4.4-sheep-manure/4.4-sheep-manure.xlsx
+++ b/packages/calculators/src/modules/test/4.4-sheep-manure/4.4-sheep-manure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/4.4-sheep-manure/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D5CFD9-019B-E042-9DC0-FA53827769D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{051355C2-0CE9-8E4B-8862-7F0738FA96B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51200" yWindow="17700" windowWidth="28800" windowHeight="25980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25205,9 +25205,11 @@
         <f>Tables!CC39</f>
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="O231">
-        <f>Tables!CC69</f>
-        <v>0.55000000000000004</v>
+      <c r="N231" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="O231" s="1">
+        <v>0.5</v>
       </c>
       <c r="Q231">
         <f>Tables!CC97</f>
@@ -25250,7 +25252,7 @@
       </c>
       <c r="AA231">
         <f t="shared" ref="AA231:AA278" si="146">(0.795*O231)-0.0014</f>
-        <v>0.43585000000000007</v>
+        <v>0.39610000000000001</v>
       </c>
       <c r="AC231">
         <f>Tables!CC168</f>
@@ -25262,15 +25264,15 @@
       </c>
       <c r="AE231">
         <f>(104.7*AA231+0.307*Q231-15)*(Q231^0.75)*10^-3</f>
-        <v>0.8646283676396137</v>
+        <v>0.78637350780019211</v>
       </c>
       <c r="AF231">
         <f>AE231*AD231*Z231</f>
-        <v>0.86462835447134123</v>
+        <v>0.7863734958237395</v>
       </c>
       <c r="AG231">
         <f t="shared" ref="AG231:AG254" si="147">(AF231 * M231) + (0.045 * X231)</f>
-        <v>6.052398481299389E-2</v>
+        <v>5.5046144707661768E-2</v>
       </c>
       <c r="AH231">
         <f t="shared" ref="AH231:AH278" si="148">$AV$2</f>
@@ -25278,7 +25280,7 @@
       </c>
       <c r="AI231">
         <f t="shared" ref="AI231:AI254" si="149">(AF231 * ((1 - O231) + (0.04 * AF231))) * ( 1 - AH231 )</f>
-        <v>0.38546716339302944</v>
+        <v>0.38448831259649313</v>
       </c>
       <c r="AJ231">
         <f t="shared" ref="AJ231:AJ278" si="150">$AV$1</f>
@@ -25290,23 +25292,23 @@
       </c>
       <c r="AL231">
         <f t="shared" ref="AL231:AL254" si="152">AI231 * AJ231 * R231 * T231 * AK231</f>
-        <v>3.0104247831031633E-4</v>
+        <v>3.0027801456951033E-4</v>
       </c>
       <c r="AM231">
         <f t="shared" ref="AM231:AM254" si="153">AI231*AJ231*S231*U231*AK231</f>
-        <v>2.3158210611975671E-4</v>
+        <v>2.3099402923392419E-4</v>
       </c>
       <c r="AN231">
         <f>AL231+AM231</f>
-        <v>5.3262458443007301E-4</v>
+        <v>5.3127204380343457E-4</v>
       </c>
       <c r="AO231">
         <f t="shared" ref="AO231:AO254" si="154">H231*AN231*L231</f>
-        <v>1.6511362117332264</v>
+        <v>1.6469433357906471</v>
       </c>
       <c r="AP231">
         <f>SUM(AO231:AO278)*10^-3</f>
-        <v>4.3988895637358368E-2</v>
+        <v>4.4522267073324906E-2</v>
       </c>
     </row>
     <row r="232" spans="1:42" x14ac:dyDescent="0.2">
@@ -25332,9 +25334,11 @@
         <f>Tables!CC39</f>
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="O232">
-        <f>Tables!CC69</f>
-        <v>0.55000000000000004</v>
+      <c r="N232" s="1">
+        <v>0.45</v>
+      </c>
+      <c r="O232" s="1">
+        <v>0.45</v>
       </c>
       <c r="Q232">
         <f>Tables!CC97</f>
@@ -25377,7 +25381,7 @@
       </c>
       <c r="AA232">
         <f t="shared" si="146"/>
-        <v>0.43585000000000007</v>
+        <v>0.35635</v>
       </c>
       <c r="AC232">
         <f>Tables!CC168</f>
@@ -25389,15 +25393,15 @@
       </c>
       <c r="AE232">
         <f t="shared" ref="AE232:AE278" si="158">(104.7*AA232+0.307*Q232-15)*(Q232^0.75)*10^-3</f>
-        <v>0.8646283676396137</v>
+        <v>0.70811864796077084</v>
       </c>
       <c r="AF232">
         <f t="shared" ref="AF232:AF278" si="159">AE232*AD232*Z232</f>
-        <v>0.86462835447134123</v>
+        <v>0.70811863717613821</v>
       </c>
       <c r="AG232">
         <f t="shared" si="147"/>
-        <v>6.052398481299389E-2</v>
+        <v>4.956830460232968E-2</v>
       </c>
       <c r="AH232">
         <f t="shared" si="148"/>
@@ -25405,7 +25409,7 @@
       </c>
       <c r="AI232">
         <f t="shared" si="149"/>
-        <v>0.38546716339302944</v>
+        <v>0.37676072816996181</v>
       </c>
       <c r="AJ232">
         <f t="shared" si="150"/>
@@ -25417,19 +25421,19 @@
       </c>
       <c r="AL232">
         <f t="shared" si="152"/>
-        <v>3.0104247831031633E-4</v>
+        <v>2.9424291900744497E-4</v>
       </c>
       <c r="AM232">
         <f t="shared" si="153"/>
-        <v>2.3158210611975671E-4</v>
+        <v>2.2635142813410056E-4</v>
       </c>
       <c r="AN232">
         <f t="shared" ref="AN232:AN254" si="160">AL232+AM232</f>
-        <v>5.3262458443007301E-4</v>
+        <v>5.2059434714154553E-4</v>
       </c>
       <c r="AO232">
         <f t="shared" si="154"/>
-        <v>1.4167813945839942</v>
+        <v>1.3847809633965111</v>
       </c>
     </row>
     <row r="233" spans="1:42" x14ac:dyDescent="0.2">
@@ -25455,9 +25459,11 @@
         <f>Tables!CC40</f>
         <v>0.13</v>
       </c>
-      <c r="O233">
-        <f>Tables!CC70</f>
-        <v>0.65</v>
+      <c r="N233" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="O233" s="1">
+        <v>0.4</v>
       </c>
       <c r="Q233">
         <f>Tables!CC98</f>
@@ -25500,7 +25506,7 @@
       </c>
       <c r="AA233">
         <f t="shared" si="146"/>
-        <v>0.51535000000000009</v>
+        <v>0.31660000000000005</v>
       </c>
       <c r="AC233">
         <f>Tables!CC169</f>
@@ -25512,15 +25518,15 @@
       </c>
       <c r="AE233">
         <f t="shared" si="158"/>
-        <v>0.97915122350076966</v>
+        <v>0.59967484520833669</v>
       </c>
       <c r="AF233">
         <f t="shared" si="159"/>
-        <v>0.97764939089749059</v>
+        <v>0.59875505752663394</v>
       </c>
       <c r="AG233">
         <f t="shared" si="147"/>
-        <v>0.12709442081667377</v>
+        <v>7.7838157478462414E-2</v>
       </c>
       <c r="AH233">
         <f t="shared" si="148"/>
@@ -25528,7 +25534,7 @@
       </c>
       <c r="AI233">
         <f t="shared" si="149"/>
-        <v>0.3499764824690102</v>
+        <v>0.3437058721307269</v>
       </c>
       <c r="AJ233">
         <f t="shared" si="150"/>
@@ -25540,19 +25546,19 @@
       </c>
       <c r="AL233">
         <f t="shared" si="152"/>
-        <v>2.7332493565832759E-4</v>
+        <v>2.6842770897852781E-4</v>
       </c>
       <c r="AM233">
         <f t="shared" si="153"/>
-        <v>2.1025990953195452E-4</v>
+        <v>2.0649263364776901E-4</v>
       </c>
       <c r="AN233">
         <f t="shared" si="160"/>
-        <v>4.8358484519028214E-4</v>
+        <v>4.7492034262629679E-4</v>
       </c>
       <c r="AO233">
         <f t="shared" si="154"/>
-        <v>1.3492017180808871</v>
+        <v>1.325027755927368</v>
       </c>
     </row>
     <row r="234" spans="1:42" x14ac:dyDescent="0.2">
@@ -25578,9 +25584,11 @@
         <f>Tables!CC40</f>
         <v>0.13</v>
       </c>
-      <c r="O234">
-        <f>Tables!CC70</f>
-        <v>0.65</v>
+      <c r="N234" s="1">
+        <v>0.45</v>
+      </c>
+      <c r="O234" s="1">
+        <v>0.45</v>
       </c>
       <c r="Q234">
         <f>Tables!CC98</f>
@@ -25623,7 +25631,7 @@
       </c>
       <c r="AA234">
         <f t="shared" si="146"/>
-        <v>0.51535000000000009</v>
+        <v>0.35635</v>
       </c>
       <c r="AC234">
         <f>Tables!CC169</f>
@@ -25635,15 +25643,15 @@
       </c>
       <c r="AE234">
         <f t="shared" si="158"/>
-        <v>0.97915122350076966</v>
+        <v>0.67557012086682311</v>
       </c>
       <c r="AF234">
         <f t="shared" si="159"/>
-        <v>0.97764939089749059</v>
+        <v>0.67453392420080505</v>
       </c>
       <c r="AG234">
         <f t="shared" si="147"/>
-        <v>0.12709442081667377</v>
+        <v>8.7689410146104665E-2</v>
       </c>
       <c r="AH234">
         <f t="shared" si="148"/>
@@ -25651,7 +25659,7 @@
       </c>
       <c r="AI234">
         <f t="shared" si="149"/>
-        <v>0.3499764824690102</v>
+        <v>0.35805801899384415</v>
       </c>
       <c r="AJ234">
         <f t="shared" si="150"/>
@@ -25663,19 +25671,19 @@
       </c>
       <c r="AL234">
         <f t="shared" si="152"/>
-        <v>2.7332493565832759E-4</v>
+        <v>2.7963646103593994E-4</v>
       </c>
       <c r="AM234">
         <f t="shared" si="153"/>
-        <v>2.1025990953195452E-4</v>
+        <v>2.1511515902358636E-4</v>
       </c>
       <c r="AN234">
         <f t="shared" si="160"/>
-        <v>4.8358484519028214E-4</v>
+        <v>4.9475162005952627E-4</v>
       </c>
       <c r="AO234">
         <f t="shared" si="154"/>
-        <v>1.8859808962421003</v>
+        <v>1.9295313182321525</v>
       </c>
     </row>
     <row r="235" spans="1:42" x14ac:dyDescent="0.2">
@@ -25701,9 +25709,11 @@
         <f>Tables!CC40</f>
         <v>0.13</v>
       </c>
-      <c r="O235">
-        <f>Tables!CC70</f>
-        <v>0.65</v>
+      <c r="N235" s="1">
+        <v>0.46</v>
+      </c>
+      <c r="O235" s="1">
+        <v>0.46</v>
       </c>
       <c r="Q235">
         <f>Tables!CC98</f>
@@ -25746,7 +25756,7 @@
       </c>
       <c r="AA235">
         <f t="shared" si="146"/>
-        <v>0.51535000000000009</v>
+        <v>0.36430000000000001</v>
       </c>
       <c r="AC235">
         <f>Tables!CC169</f>
@@ -25758,15 +25768,15 @@
       </c>
       <c r="AE235">
         <f t="shared" si="158"/>
-        <v>0.97915122350076966</v>
+        <v>0.69074917599852059</v>
       </c>
       <c r="AF235">
         <f t="shared" si="159"/>
-        <v>0.97764939089749059</v>
+        <v>0.68968969753563947</v>
       </c>
       <c r="AG235">
         <f t="shared" si="147"/>
-        <v>0.19909442081667378</v>
+        <v>0.16165966067963311</v>
       </c>
       <c r="AH235">
         <f t="shared" si="148"/>
@@ -25774,7 +25784,7 @@
       </c>
       <c r="AI235">
         <f t="shared" si="149"/>
-        <v>0.3499764824690102</v>
+        <v>0.36014256687874002</v>
       </c>
       <c r="AJ235">
         <f t="shared" si="150"/>
@@ -25786,19 +25796,19 @@
       </c>
       <c r="AL235">
         <f t="shared" si="152"/>
-        <v>2.7332493565832759E-4</v>
+        <v>2.8126445304413528E-4</v>
       </c>
       <c r="AM235">
         <f t="shared" si="153"/>
-        <v>2.1025990953195452E-4</v>
+        <v>2.1636751988681109E-4</v>
       </c>
       <c r="AN235">
         <f t="shared" si="160"/>
-        <v>4.8358484519028214E-4</v>
+        <v>4.9763197293094643E-4</v>
       </c>
       <c r="AO235">
         <f t="shared" si="154"/>
-        <v>1.9488469261168369</v>
+        <v>2.0054568509117141</v>
       </c>
     </row>
     <row r="236" spans="1:42" x14ac:dyDescent="0.2">
@@ -25827,9 +25837,11 @@
         <f>Tables!CC41</f>
         <v>0.1</v>
       </c>
-      <c r="O236">
-        <f>Tables!CC71</f>
-        <v>0.6</v>
+      <c r="N236" s="1">
+        <v>0.51</v>
+      </c>
+      <c r="O236" s="1">
+        <v>0.51</v>
       </c>
       <c r="Q236">
         <f>Tables!CC99</f>
@@ -25872,7 +25884,7 @@
       </c>
       <c r="AA236">
         <f t="shared" si="146"/>
-        <v>0.47559999999999997</v>
+        <v>0.40405000000000002</v>
       </c>
       <c r="AC236">
         <f>Tables!CC170</f>
@@ -25884,15 +25896,15 @@
       </c>
       <c r="AE236">
         <f t="shared" si="158"/>
-        <v>0.84457430670543054</v>
+        <v>0.71441785360642229</v>
       </c>
       <c r="AF236">
         <f t="shared" si="159"/>
-        <v>0.73027360369308525</v>
+        <v>0.61773191103930425</v>
       </c>
       <c r="AG236">
         <f t="shared" si="147"/>
-        <v>7.3027360369308528E-2</v>
+        <v>6.1773191103930425E-2</v>
       </c>
       <c r="AH236">
         <f t="shared" si="148"/>
@@ -25900,7 +25912,7 @@
       </c>
       <c r="AI236">
         <f t="shared" si="149"/>
-        <v>0.28836610909308796</v>
+        <v>0.29251615736863712</v>
       </c>
       <c r="AJ236">
         <f t="shared" si="150"/>
@@ -25912,19 +25924,19 @@
       </c>
       <c r="AL236">
         <f t="shared" si="152"/>
-        <v>2.2520841302783737E-4</v>
+        <v>2.2844952131571749E-4</v>
       </c>
       <c r="AM236">
         <f t="shared" si="153"/>
-        <v>1.7324544661472571E-4</v>
+        <v>1.7573872493106937E-4</v>
       </c>
       <c r="AN236">
         <f t="shared" si="160"/>
-        <v>3.9845385964256308E-4</v>
+        <v>4.0418824624678684E-4</v>
       </c>
       <c r="AO236">
         <f t="shared" si="154"/>
-        <v>1.2451683113830097</v>
+        <v>1.2630882695212089</v>
       </c>
     </row>
     <row r="237" spans="1:42" x14ac:dyDescent="0.2">
@@ -25950,9 +25962,11 @@
         <f>Tables!CC41</f>
         <v>0.1</v>
       </c>
-      <c r="O237">
-        <f>Tables!CC71</f>
-        <v>0.6</v>
+      <c r="N237" s="1">
+        <v>0.45</v>
+      </c>
+      <c r="O237" s="1">
+        <v>0.45</v>
       </c>
       <c r="Q237">
         <f>Tables!CC99</f>
@@ -25995,7 +26009,7 @@
       </c>
       <c r="AA237">
         <f t="shared" si="146"/>
-        <v>0.47559999999999997</v>
+        <v>0.35635</v>
       </c>
       <c r="AC237">
         <f>Tables!CC170</f>
@@ -26007,15 +26021,15 @@
       </c>
       <c r="AE237">
         <f t="shared" si="158"/>
-        <v>0.84457430670543054</v>
+        <v>0.62764688487374998</v>
       </c>
       <c r="AF237">
         <f t="shared" si="159"/>
-        <v>0.73027360369308525</v>
+        <v>0.54270411593678336</v>
       </c>
       <c r="AG237">
         <f t="shared" si="147"/>
-        <v>7.3027360369308528E-2</v>
+        <v>5.427041159367834E-2</v>
       </c>
       <c r="AH237">
         <f t="shared" si="148"/>
@@ -26023,7 +26037,7 @@
       </c>
       <c r="AI237">
         <f t="shared" si="149"/>
-        <v>0.28836610909308796</v>
+        <v>0.28544690413834639</v>
       </c>
       <c r="AJ237">
         <f t="shared" si="150"/>
@@ -26035,19 +26049,19 @@
       </c>
       <c r="AL237">
         <f t="shared" si="152"/>
-        <v>2.2520841302783737E-4</v>
+        <v>2.2292856982009026E-4</v>
       </c>
       <c r="AM237">
         <f t="shared" si="153"/>
-        <v>1.7324544661472571E-4</v>
+        <v>1.7149163800061823E-4</v>
       </c>
       <c r="AN237">
         <f t="shared" si="160"/>
-        <v>3.9845385964256308E-4</v>
+        <v>3.9442020782070849E-4</v>
       </c>
       <c r="AO237">
         <f t="shared" si="154"/>
-        <v>1.4822483578703347</v>
+        <v>1.4672431730930358</v>
       </c>
     </row>
     <row r="238" spans="1:42" x14ac:dyDescent="0.2">
@@ -26073,9 +26087,11 @@
         <f>Tables!CC41</f>
         <v>0.1</v>
       </c>
-      <c r="O238">
-        <f>Tables!CC71</f>
-        <v>0.6</v>
+      <c r="N238" s="1">
+        <v>0.44</v>
+      </c>
+      <c r="O238" s="1">
+        <v>0.44</v>
       </c>
       <c r="Q238">
         <f>Tables!CC99</f>
@@ -26118,7 +26134,7 @@
       </c>
       <c r="AA238">
         <f t="shared" si="146"/>
-        <v>0.47559999999999997</v>
+        <v>0.34839999999999999</v>
       </c>
       <c r="AC238">
         <f>Tables!CC170</f>
@@ -26130,15 +26146,15 @@
       </c>
       <c r="AE238">
         <f t="shared" si="158"/>
-        <v>0.84457430670543054</v>
+        <v>0.61318505675163781</v>
       </c>
       <c r="AF238">
         <f t="shared" si="159"/>
-        <v>0.73027360369308525</v>
+        <v>0.53019948341969647</v>
       </c>
       <c r="AG238">
         <f t="shared" si="147"/>
-        <v>7.3027360369308528E-2</v>
+        <v>5.3019948341969651E-2</v>
       </c>
       <c r="AH238">
         <f t="shared" si="148"/>
@@ -26146,7 +26162,7 @@
       </c>
       <c r="AI238">
         <f t="shared" si="149"/>
-        <v>0.28836610909308796</v>
+        <v>0.28350367677146893</v>
       </c>
       <c r="AJ238">
         <f t="shared" si="150"/>
@@ -26158,19 +26174,19 @@
       </c>
       <c r="AL238">
         <f t="shared" si="152"/>
-        <v>2.2520841302783737E-4</v>
+        <v>2.2141094643215781E-4</v>
       </c>
       <c r="AM238">
         <f t="shared" si="153"/>
-        <v>1.7324544661472571E-4</v>
+        <v>1.7032418009751223E-4</v>
       </c>
       <c r="AN238">
         <f t="shared" si="160"/>
-        <v>3.9845385964256308E-4</v>
+        <v>3.9173512652967003E-4</v>
       </c>
       <c r="AO238">
         <f t="shared" si="154"/>
-        <v>1.4204880096257373</v>
+        <v>1.3965357260782736</v>
       </c>
     </row>
     <row r="239" spans="1:42" x14ac:dyDescent="0.2">
@@ -26199,9 +26215,11 @@
         <f>Tables!CC38</f>
         <v>0.16</v>
       </c>
-      <c r="O239">
-        <f>Tables!CC68</f>
-        <v>0.7</v>
+      <c r="N239" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="O239" s="1">
+        <v>0.65</v>
       </c>
       <c r="Q239">
         <f>Tables!CC96</f>
@@ -26244,7 +26262,7 @@
       </c>
       <c r="AA239">
         <f t="shared" si="146"/>
-        <v>0.55510000000000004</v>
+        <v>0.51535000000000009</v>
       </c>
       <c r="AC239">
         <f>Tables!CC167</f>
@@ -26256,15 +26274,15 @@
       </c>
       <c r="AE239">
         <f t="shared" si="158"/>
-        <v>1.2118587484135388</v>
+        <v>1.1278052426935643</v>
       </c>
       <c r="AF239">
         <f t="shared" si="159"/>
-        <v>1.2444335099837347</v>
+        <v>1.1581206461400915</v>
       </c>
       <c r="AG239">
         <f t="shared" si="147"/>
-        <v>0.19910936159739756</v>
+        <v>0.18529930338241463</v>
       </c>
       <c r="AH239">
         <f t="shared" si="148"/>
@@ -26272,7 +26290,7 @@
       </c>
       <c r="AI239">
         <f t="shared" si="149"/>
-        <v>0.40045267195186296</v>
+        <v>0.42227260631849611</v>
       </c>
       <c r="AJ239">
         <f t="shared" si="150"/>
@@ -26284,19 +26302,19 @@
       </c>
       <c r="AL239">
         <f t="shared" si="152"/>
-        <v>3.1274587373207352E-4</v>
+        <v>3.2978682492614995E-4</v>
       </c>
       <c r="AM239">
         <f t="shared" si="153"/>
-        <v>2.4058514441433607E-4</v>
+        <v>2.5369418932374001E-4</v>
       </c>
       <c r="AN239">
         <f t="shared" si="160"/>
-        <v>5.5333101814640962E-4</v>
+        <v>5.8348101424988996E-4</v>
       </c>
       <c r="AO239">
         <f t="shared" si="154"/>
-        <v>1.4607938879065214</v>
+        <v>1.5403898776197096</v>
       </c>
     </row>
     <row r="240" spans="1:42" x14ac:dyDescent="0.2">
@@ -26322,9 +26340,11 @@
         <f>Tables!CC38</f>
         <v>0.16</v>
       </c>
-      <c r="O240">
-        <f>Tables!CC68</f>
-        <v>0.7</v>
+      <c r="N240" s="1">
+        <v>0.66</v>
+      </c>
+      <c r="O240" s="1">
+        <v>0.66</v>
       </c>
       <c r="Q240">
         <f>Tables!CC96</f>
@@ -26367,7 +26387,7 @@
       </c>
       <c r="AA240">
         <f t="shared" si="146"/>
-        <v>0.55510000000000004</v>
+        <v>0.5233000000000001</v>
       </c>
       <c r="AC240">
         <f>Tables!CC167</f>
@@ -26379,15 +26399,15 @@
       </c>
       <c r="AE240">
         <f t="shared" si="158"/>
-        <v>1.2118587484135388</v>
+        <v>1.1446159438375592</v>
       </c>
       <c r="AF240">
         <f t="shared" si="159"/>
-        <v>1.2423975872889967</v>
+        <v>1.1734602641256255</v>
       </c>
       <c r="AG240">
         <f t="shared" si="147"/>
-        <v>0.19878361396623948</v>
+        <v>0.18775364226010008</v>
       </c>
       <c r="AH240">
         <f t="shared" si="148"/>
@@ -26395,7 +26415,7 @@
       </c>
       <c r="AI240">
         <f t="shared" si="149"/>
-        <v>0.39970443904013914</v>
+        <v>0.41773230150502522</v>
       </c>
       <c r="AJ240">
         <f t="shared" si="150"/>
@@ -26407,19 +26427,19 @@
       </c>
       <c r="AL240">
         <f t="shared" si="152"/>
-        <v>3.121615181462022E-4</v>
+        <v>3.2624093375010213E-4</v>
       </c>
       <c r="AM240">
         <f t="shared" si="153"/>
-        <v>2.401356188255936E-4</v>
+        <v>2.5096645152663692E-4</v>
       </c>
       <c r="AN240">
         <f t="shared" si="160"/>
-        <v>5.5229713697179576E-4</v>
+        <v>5.7720738527673905E-4</v>
       </c>
       <c r="AO240">
         <f t="shared" si="154"/>
-        <v>1.7977271808431952</v>
+        <v>1.8788100390757856</v>
       </c>
     </row>
     <row r="241" spans="5:41" x14ac:dyDescent="0.2">
@@ -26445,9 +26465,11 @@
         <f>Tables!CC38</f>
         <v>0.16</v>
       </c>
-      <c r="O241">
-        <f>Tables!CC68</f>
-        <v>0.7</v>
+      <c r="N241" s="1">
+        <v>0.62</v>
+      </c>
+      <c r="O241" s="1">
+        <v>0.62</v>
       </c>
       <c r="Q241">
         <f>Tables!CC96</f>
@@ -26490,7 +26512,7 @@
       </c>
       <c r="AA241">
         <f t="shared" si="146"/>
-        <v>0.55510000000000004</v>
+        <v>0.49149999999999999</v>
       </c>
       <c r="AC241">
         <f>Tables!CC167</f>
@@ -26502,15 +26524,15 @@
       </c>
       <c r="AE241">
         <f t="shared" si="158"/>
-        <v>1.2118587484135388</v>
+        <v>1.0773731392615793</v>
       </c>
       <c r="AF241">
         <f t="shared" si="159"/>
-        <v>1.2525772007626874</v>
+        <v>1.113572875320509</v>
       </c>
       <c r="AG241">
         <f t="shared" si="147"/>
-        <v>0.20041235212202999</v>
+        <v>0.17817166005128143</v>
       </c>
       <c r="AH241">
         <f t="shared" si="148"/>
@@ -26518,7 +26540,7 @@
       </c>
       <c r="AI241">
         <f t="shared" si="149"/>
-        <v>0.40344865430493582</v>
+        <v>0.43493871660235472</v>
       </c>
       <c r="AJ241">
         <f t="shared" si="150"/>
@@ -26530,19 +26552,19 @@
       </c>
       <c r="AL241">
         <f t="shared" si="152"/>
-        <v>3.1508567861870512E-4</v>
+        <v>3.3967881467915708E-4</v>
       </c>
       <c r="AM241">
         <f t="shared" si="153"/>
-        <v>2.4238507958161465E-4</v>
+        <v>2.6130377264093241E-4</v>
       </c>
       <c r="AN241">
         <f t="shared" si="160"/>
-        <v>5.5747075820031982E-4</v>
+        <v>6.0098258732008949E-4</v>
       </c>
       <c r="AO241">
         <f t="shared" si="154"/>
-        <v>1.7560328883310075</v>
+        <v>1.893095150058282</v>
       </c>
     </row>
     <row r="242" spans="5:41" x14ac:dyDescent="0.2">
@@ -26568,9 +26590,11 @@
         <f>Tables!CC39</f>
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="O242">
-        <f>Tables!CC69</f>
-        <v>0.55000000000000004</v>
+      <c r="N242" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="O242" s="1">
+        <v>0.6</v>
       </c>
       <c r="Q242">
         <f>Tables!CC97</f>
@@ -26613,7 +26637,7 @@
       </c>
       <c r="AA242">
         <f t="shared" si="146"/>
-        <v>0.43585000000000007</v>
+        <v>0.47559999999999997</v>
       </c>
       <c r="AC242">
         <f>Tables!CC168</f>
@@ -26625,15 +26649,15 @@
       </c>
       <c r="AE242">
         <f t="shared" si="158"/>
-        <v>0.8646283676396137</v>
+        <v>0.94288322747903475</v>
       </c>
       <c r="AF242">
         <f t="shared" si="159"/>
-        <v>0.86462835447134123</v>
+        <v>0.9428832131189423</v>
       </c>
       <c r="AG242">
         <f t="shared" si="147"/>
-        <v>6.052398481299389E-2</v>
+        <v>6.6001824918325971E-2</v>
       </c>
       <c r="AH242">
         <f t="shared" si="148"/>
@@ -26641,7 +26665,7 @@
       </c>
       <c r="AI242">
         <f t="shared" si="149"/>
-        <v>0.38546716339302944</v>
+        <v>0.37969728055957003</v>
       </c>
       <c r="AJ242">
         <f t="shared" si="150"/>
@@ -26653,19 +26677,19 @@
       </c>
       <c r="AL242">
         <f t="shared" si="152"/>
-        <v>3.0104247831031633E-4</v>
+        <v>2.9653631022986249E-4</v>
       </c>
       <c r="AM242">
         <f t="shared" si="153"/>
-        <v>2.3158210611975671E-4</v>
+        <v>2.2811565879159781E-4</v>
       </c>
       <c r="AN242">
         <f t="shared" si="160"/>
-        <v>5.3262458443007301E-4</v>
+        <v>5.246519690214603E-4</v>
       </c>
       <c r="AO242">
         <f t="shared" si="154"/>
-        <v>1.6511362117332264</v>
+        <v>1.6264211039665268</v>
       </c>
     </row>
     <row r="243" spans="5:41" x14ac:dyDescent="0.2">
@@ -26741,13 +26765,15 @@
         <f t="shared" si="146"/>
         <v>0.43585000000000007</v>
       </c>
-      <c r="AC243">
-        <f>Tables!CC172</f>
-        <v>3</v>
+      <c r="AB243" s="1">
+        <v>2.8</v>
+      </c>
+      <c r="AC243" s="1">
+        <v>2.8</v>
       </c>
       <c r="AD243">
         <f t="shared" si="157"/>
-        <v>0.99999998477002028</v>
+        <v>0.99999984502468642</v>
       </c>
       <c r="AE243">
         <f t="shared" si="158"/>
@@ -26755,11 +26781,11 @@
       </c>
       <c r="AF243">
         <f t="shared" si="159"/>
-        <v>0.47750864035368012</v>
+        <v>0.47750857362407473</v>
       </c>
       <c r="AG243">
         <f t="shared" si="147"/>
-        <v>3.3425604824757614E-2</v>
+        <v>3.3425600153685231E-2</v>
       </c>
       <c r="AH243">
         <f t="shared" si="148"/>
@@ -26767,7 +26793,7 @@
       </c>
       <c r="AI243">
         <f t="shared" si="149"/>
-        <v>0.20607951076576064</v>
+        <v>0.20607948079451649</v>
       </c>
       <c r="AJ243">
         <f t="shared" si="150"/>
@@ -26779,19 +26805,19 @@
       </c>
       <c r="AL243">
         <f t="shared" si="152"/>
-        <v>1.6094415437054054E-4</v>
+        <v>1.6094413096357239E-4</v>
       </c>
       <c r="AM243">
         <f t="shared" si="153"/>
-        <v>1.238090599240053E-4</v>
+        <v>1.2380904191779232E-4</v>
       </c>
       <c r="AN243">
         <f t="shared" si="160"/>
-        <v>2.8475321429454587E-4</v>
+        <v>2.8475317288136472E-4</v>
       </c>
       <c r="AO243">
         <f>H243*AN243*L243</f>
-        <v>0.35309398572523687</v>
+        <v>0.35309393437289222</v>
       </c>
     </row>
     <row r="244" spans="5:41" x14ac:dyDescent="0.2">
@@ -26864,13 +26890,15 @@
         <f t="shared" si="146"/>
         <v>0.43585000000000007</v>
       </c>
-      <c r="AC244">
-        <f>Tables!CC172</f>
-        <v>3</v>
+      <c r="AB244" s="1">
+        <v>2.7</v>
+      </c>
+      <c r="AC244" s="1">
+        <v>2.7</v>
       </c>
       <c r="AD244">
         <f t="shared" si="157"/>
-        <v>0.99999998477002028</v>
+        <v>0.99999953442842837</v>
       </c>
       <c r="AE244">
         <f t="shared" si="158"/>
@@ -26878,11 +26906,11 @@
       </c>
       <c r="AF244">
         <f t="shared" si="159"/>
-        <v>0.47750864035368012</v>
+        <v>0.47750842531167564</v>
       </c>
       <c r="AG244">
         <f t="shared" si="147"/>
-        <v>3.3425604824757614E-2</v>
+        <v>3.3425589771817296E-2</v>
       </c>
       <c r="AH244">
         <f t="shared" si="148"/>
@@ -26890,7 +26918,7 @@
       </c>
       <c r="AI244">
         <f t="shared" si="149"/>
-        <v>0.20607951076576064</v>
+        <v>0.20607941418079953</v>
       </c>
       <c r="AJ244">
         <f t="shared" si="150"/>
@@ -26902,19 +26930,19 @@
       </c>
       <c r="AL244">
         <f t="shared" si="152"/>
-        <v>1.6094415437054054E-4</v>
+        <v>1.6094407893953419E-4</v>
       </c>
       <c r="AM244">
         <f t="shared" si="153"/>
-        <v>1.238090599240053E-4</v>
+        <v>1.238090018974058E-4</v>
       </c>
       <c r="AN244">
         <f t="shared" si="160"/>
-        <v>2.8475321429454587E-4</v>
+        <v>2.8475308083694001E-4</v>
       </c>
       <c r="AO244">
         <f t="shared" si="154"/>
-        <v>0.31892360000989139</v>
+        <v>0.31892345053737281</v>
       </c>
     </row>
     <row r="245" spans="5:41" x14ac:dyDescent="0.2">
@@ -26987,13 +27015,15 @@
         <f t="shared" si="146"/>
         <v>0.51535000000000009</v>
       </c>
-      <c r="AC245">
-        <f>Tables!CC173</f>
-        <v>1.8</v>
+      <c r="AB245" s="1">
+        <v>2.4</v>
+      </c>
+      <c r="AC245" s="1">
+        <v>2.4</v>
       </c>
       <c r="AD245">
         <f t="shared" si="157"/>
-        <v>0.99846618932067555</v>
+        <v>0.99999007049569411</v>
       </c>
       <c r="AE245">
         <f t="shared" si="158"/>
@@ -27001,11 +27031,11 @@
       </c>
       <c r="AF245">
         <f t="shared" si="159"/>
-        <v>0.67483164337990365</v>
+        <v>0.67586158635509153</v>
       </c>
       <c r="AG245">
         <f t="shared" si="147"/>
-        <v>8.772811363938747E-2</v>
+        <v>8.7862006226161901E-2</v>
       </c>
       <c r="AH245">
         <f t="shared" si="148"/>
@@ -27013,7 +27043,7 @@
       </c>
       <c r="AI245">
         <f t="shared" si="149"/>
-        <v>0.23405442625450001</v>
+        <v>0.23443726173424295</v>
       </c>
       <c r="AJ245">
         <f t="shared" si="150"/>
@@ -27025,19 +27055,19 @@
       </c>
       <c r="AL245">
         <f t="shared" si="152"/>
-        <v>1.8279202803926314E-4</v>
+        <v>1.8309101522300263E-4</v>
       </c>
       <c r="AM245">
         <f t="shared" si="153"/>
-        <v>1.4061591265402342E-4</v>
+        <v>1.4084591368943155E-4</v>
       </c>
       <c r="AN245">
         <f t="shared" si="160"/>
-        <v>3.2340794069328656E-4</v>
+        <v>3.2393692891243421E-4</v>
       </c>
       <c r="AO245">
         <f t="shared" si="154"/>
-        <v>0.40102584645967537</v>
+        <v>0.40168179185141845</v>
       </c>
     </row>
     <row r="246" spans="5:41" x14ac:dyDescent="0.2">
@@ -27110,13 +27140,15 @@
         <f t="shared" si="146"/>
         <v>0.51535000000000009</v>
       </c>
-      <c r="AC246">
-        <f>Tables!CC173</f>
-        <v>1.8</v>
+      <c r="AB246" s="1">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="AC246" s="1">
+        <v>2.2000000000000002</v>
       </c>
       <c r="AD246">
         <f t="shared" si="157"/>
-        <v>0.99846618932067555</v>
+        <v>0.99993747849622516</v>
       </c>
       <c r="AE246">
         <f t="shared" si="158"/>
@@ -27124,11 +27156,11 @@
       </c>
       <c r="AF246">
         <f t="shared" si="159"/>
-        <v>0.67483164337990365</v>
+        <v>0.67582604108995403</v>
       </c>
       <c r="AG246">
         <f t="shared" si="147"/>
-        <v>8.772811363938747E-2</v>
+        <v>8.785738534169403E-2</v>
       </c>
       <c r="AH246">
         <f t="shared" si="148"/>
@@ -27136,7 +27168,7 @@
       </c>
       <c r="AI246">
         <f t="shared" si="149"/>
-        <v>0.23405442625450001</v>
+        <v>0.23442404806256897</v>
       </c>
       <c r="AJ246">
         <f t="shared" si="150"/>
@@ -27148,19 +27180,19 @@
       </c>
       <c r="AL246">
         <f t="shared" si="152"/>
-        <v>1.8279202803926314E-4</v>
+        <v>1.8308069559828209E-4</v>
       </c>
       <c r="AM246">
         <f t="shared" si="153"/>
-        <v>1.4061591265402342E-4</v>
+        <v>1.4083797514055776E-4</v>
       </c>
       <c r="AN246">
         <f t="shared" si="160"/>
-        <v>3.2340794069328656E-4</v>
+        <v>3.2391867073883987E-4</v>
       </c>
       <c r="AO246">
         <f t="shared" si="154"/>
-        <v>0.33957833772795087</v>
+        <v>0.34011460427578188</v>
       </c>
     </row>
     <row r="247" spans="5:41" x14ac:dyDescent="0.2">
@@ -27233,13 +27265,15 @@
         <f t="shared" si="146"/>
         <v>0.51535000000000009</v>
       </c>
-      <c r="AC247">
-        <f>Tables!CC173</f>
-        <v>1.8</v>
+      <c r="AB247" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="AC247" s="1">
+        <v>1.9</v>
       </c>
       <c r="AD247">
         <f t="shared" si="157"/>
-        <v>0.99846618932067555</v>
+        <v>0.99926819758111951</v>
       </c>
       <c r="AE247">
         <f t="shared" si="158"/>
@@ -27247,11 +27281,11 @@
       </c>
       <c r="AF247">
         <f t="shared" si="159"/>
-        <v>0.67483164337990365</v>
+        <v>0.67537369533738445</v>
       </c>
       <c r="AG247">
         <f t="shared" si="147"/>
-        <v>8.772811363938747E-2</v>
+        <v>8.7798580393859987E-2</v>
       </c>
       <c r="AH247">
         <f t="shared" si="148"/>
@@ -27259,7 +27293,7 @@
       </c>
       <c r="AI247">
         <f t="shared" si="149"/>
-        <v>0.23405442625450001</v>
+        <v>0.234255900222053</v>
       </c>
       <c r="AJ247">
         <f t="shared" si="150"/>
@@ -27271,19 +27305,19 @@
       </c>
       <c r="AL247">
         <f t="shared" si="152"/>
-        <v>1.8279202803926314E-4</v>
+        <v>1.8294937535251617E-4</v>
       </c>
       <c r="AM247">
         <f t="shared" si="153"/>
-        <v>1.4061591265402342E-4</v>
+        <v>1.4073695478203119E-4</v>
       </c>
       <c r="AN247">
         <f t="shared" si="160"/>
-        <v>3.2340794069328656E-4</v>
+        <v>3.2368633013454736E-4</v>
       </c>
       <c r="AO247">
         <f t="shared" si="154"/>
-        <v>0.35089761565221594</v>
+        <v>0.35119966819598386</v>
       </c>
     </row>
     <row r="248" spans="5:41" x14ac:dyDescent="0.2">
@@ -27356,13 +27390,15 @@
         <f t="shared" si="146"/>
         <v>0.47559999999999997</v>
       </c>
-      <c r="AC248">
-        <f>Tables!CC174</f>
-        <v>1</v>
+      <c r="AB248" s="1">
+        <v>1.4</v>
+      </c>
+      <c r="AC248" s="1">
+        <v>1.4</v>
       </c>
       <c r="AD248">
         <f t="shared" si="157"/>
-        <v>0.8646647167633873</v>
+        <v>0.98015890525562965</v>
       </c>
       <c r="AE248">
         <f t="shared" si="158"/>
@@ -27370,11 +27406,11 @@
       </c>
       <c r="AF248">
         <f t="shared" si="159"/>
-        <v>0.56662384770561869</v>
+        <v>0.6423083994195754</v>
       </c>
       <c r="AG248">
         <f t="shared" si="147"/>
-        <v>5.6662384770561874E-2</v>
+        <v>6.4230839941957538E-2</v>
       </c>
       <c r="AH248">
         <f t="shared" si="148"/>
@@ -27382,7 +27418,7 @@
       </c>
       <c r="AI248">
         <f t="shared" si="149"/>
-        <v>0.2203326790758926</v>
+        <v>0.25155170192911341</v>
       </c>
       <c r="AJ248">
         <f t="shared" si="150"/>
@@ -27394,19 +27430,19 @@
       </c>
       <c r="AL248">
         <f t="shared" si="152"/>
-        <v>1.720756060721248E-4</v>
+        <v>1.9645706551326883E-4</v>
       </c>
       <c r="AM248">
         <f t="shared" si="153"/>
-        <v>1.3237212067108688E-4</v>
+        <v>1.5112797784893445E-4</v>
       </c>
       <c r="AN248">
         <f t="shared" si="160"/>
-        <v>3.0444772674321168E-4</v>
+        <v>3.4758504336220329E-4</v>
       </c>
       <c r="AO248">
         <f t="shared" si="154"/>
-        <v>0.3196701130803723</v>
+        <v>0.36496429553031345</v>
       </c>
     </row>
     <row r="249" spans="5:41" x14ac:dyDescent="0.2">
@@ -27479,13 +27515,15 @@
         <f t="shared" si="146"/>
         <v>0.47559999999999997</v>
       </c>
-      <c r="AC249">
-        <f>Tables!CC174</f>
-        <v>1</v>
+      <c r="AB249" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="AC249" s="1">
+        <v>1.3</v>
       </c>
       <c r="AD249">
         <f t="shared" si="157"/>
-        <v>0.8646647167633873</v>
+        <v>0.96595254526540064</v>
       </c>
       <c r="AE249">
         <f t="shared" si="158"/>
@@ -27493,11 +27531,11 @@
       </c>
       <c r="AF249">
         <f t="shared" si="159"/>
-        <v>0.56662384770561869</v>
+        <v>0.63299882288257248</v>
       </c>
       <c r="AG249">
         <f t="shared" si="147"/>
-        <v>5.6662384770561874E-2</v>
+        <v>6.3299882288257253E-2</v>
       </c>
       <c r="AH249">
         <f t="shared" si="148"/>
@@ -27505,7 +27543,7 @@
       </c>
       <c r="AI249">
         <f t="shared" si="149"/>
-        <v>0.2203326790758926</v>
+        <v>0.2476888671803493</v>
       </c>
       <c r="AJ249">
         <f t="shared" si="150"/>
@@ -27517,19 +27555,19 @@
       </c>
       <c r="AL249">
         <f t="shared" si="152"/>
-        <v>1.720756060721248E-4</v>
+        <v>1.9344026549368985E-4</v>
       </c>
       <c r="AM249">
         <f t="shared" si="153"/>
-        <v>1.3237212067108688E-4</v>
+        <v>1.4880725252738674E-4</v>
       </c>
       <c r="AN249">
         <f t="shared" si="160"/>
-        <v>3.0444772674321168E-4</v>
+        <v>3.4224751802107661E-4</v>
       </c>
       <c r="AO249">
         <f t="shared" si="154"/>
-        <v>0.75503036232316489</v>
+        <v>0.84877384469226991</v>
       </c>
     </row>
     <row r="250" spans="5:41" x14ac:dyDescent="0.2">
@@ -27602,13 +27640,15 @@
         <f t="shared" si="146"/>
         <v>0.47559999999999997</v>
       </c>
-      <c r="AC250">
-        <f>Tables!CC174</f>
-        <v>1</v>
+      <c r="AB250" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AC250" s="1">
+        <v>1.1000000000000001</v>
       </c>
       <c r="AD250">
         <f t="shared" si="157"/>
-        <v>0.8646647167633873</v>
+        <v>0.91107838254061368</v>
       </c>
       <c r="AE250">
         <f t="shared" si="158"/>
@@ -27616,11 +27656,11 @@
       </c>
       <c r="AF250">
         <f t="shared" si="159"/>
-        <v>0.56662384770561869</v>
+        <v>0.59703920915029218</v>
       </c>
       <c r="AG250">
         <f t="shared" si="147"/>
-        <v>5.6662384770561874E-2</v>
+        <v>5.970392091502922E-2</v>
       </c>
       <c r="AH250">
         <f t="shared" si="148"/>
@@ -27628,7 +27668,7 @@
       </c>
       <c r="AI250">
         <f t="shared" si="149"/>
-        <v>0.2203326790758926</v>
+        <v>0.23282800304257883</v>
       </c>
       <c r="AJ250">
         <f t="shared" si="150"/>
@@ -27640,19 +27680,19 @@
       </c>
       <c r="AL250">
         <f t="shared" si="152"/>
-        <v>1.720756060721248E-4</v>
+        <v>1.8183421497958729E-4</v>
       </c>
       <c r="AM250">
         <f t="shared" si="153"/>
-        <v>1.3237212067108688E-4</v>
+        <v>1.3987909847791867E-4</v>
       </c>
       <c r="AN250">
         <f t="shared" si="160"/>
-        <v>3.0444772674321168E-4</v>
+        <v>3.2171331345750599E-4</v>
       </c>
       <c r="AO250">
         <f t="shared" si="154"/>
-        <v>0.84940915761356062</v>
+        <v>0.89758014454644175</v>
       </c>
     </row>
     <row r="251" spans="5:41" x14ac:dyDescent="0.2">
@@ -28180,9 +28220,11 @@
         <f>Tables!CC85</f>
         <v>0.55000000000000004</v>
       </c>
-      <c r="Q255">
-        <f>Tables!CC113</f>
-        <v>65</v>
+      <c r="P255" s="1">
+        <v>66</v>
+      </c>
+      <c r="Q255" s="1">
+        <v>66</v>
       </c>
       <c r="R255">
         <f>$R$231</f>
@@ -28233,15 +28275,15 @@
       </c>
       <c r="AE255">
         <f t="shared" si="158"/>
-        <v>1.1580752413958724</v>
+        <v>1.1785209149153895</v>
       </c>
       <c r="AF255">
         <f t="shared" si="159"/>
-        <v>1.15807522375841</v>
+        <v>1.1785208969665397</v>
       </c>
       <c r="AG255">
         <f t="shared" ref="AG255:AG278" si="161">(AF255 * M255) + (0.045 * X255)</f>
-        <v>8.1065265663088706E-2</v>
+        <v>8.2496462787657793E-2</v>
       </c>
       <c r="AH255">
         <f t="shared" si="148"/>
@@ -28249,7 +28291,7 @@
       </c>
       <c r="AI255">
         <f t="shared" ref="AI255:AI278" si="162">(AF255 * ((1 - O255) + (0.04 * AF255))) * ( 1 - AH255 )</f>
-        <v>0.52879702927487948</v>
+        <v>0.53901959471294225</v>
       </c>
       <c r="AJ255">
         <f t="shared" si="150"/>
@@ -28261,19 +28303,19 @@
       </c>
       <c r="AL255">
         <f t="shared" ref="AL255:AL278" si="163">AI255 * AJ255 * R255 * T255 * AK255</f>
-        <v>4.1298036080372741E-4</v>
+        <v>4.2096398879184219E-4</v>
       </c>
       <c r="AM255">
         <f t="shared" ref="AM255:AM278" si="164">AI255*AJ255*S255*U255*AK255</f>
-        <v>3.1769224820969987E-4</v>
+        <v>3.2383379140433978E-4</v>
       </c>
       <c r="AN255">
         <f t="shared" ref="AN255:AN278" si="165">AL255+AM255</f>
-        <v>7.3067260901342728E-4</v>
+        <v>7.4479778019618192E-4</v>
       </c>
       <c r="AO255">
         <f t="shared" ref="AO255:AO278" si="166">H255*AN255*L255</f>
-        <v>0.45301701758832491</v>
+        <v>0.4617746237216328</v>
       </c>
     </row>
     <row r="256" spans="5:41" x14ac:dyDescent="0.2">
@@ -28303,9 +28345,11 @@
         <f>Tables!CC85</f>
         <v>0.55000000000000004</v>
       </c>
-      <c r="Q256">
-        <f>Tables!CC113</f>
-        <v>65</v>
+      <c r="P256" s="1">
+        <v>67</v>
+      </c>
+      <c r="Q256" s="1">
+        <v>67</v>
       </c>
       <c r="R256">
         <f>$R$231</f>
@@ -28356,15 +28400,15 @@
       </c>
       <c r="AE256">
         <f t="shared" si="158"/>
-        <v>1.1580752413958724</v>
+        <v>1.199077422939921</v>
       </c>
       <c r="AF256">
         <f t="shared" si="159"/>
-        <v>1.15807522375841</v>
+        <v>1.1990774046779962</v>
       </c>
       <c r="AG256">
         <f t="shared" si="161"/>
-        <v>8.1065265663088706E-2</v>
+        <v>8.3935418327459738E-2</v>
       </c>
       <c r="AH256">
         <f t="shared" si="148"/>
@@ -28372,7 +28416,7 @@
       </c>
       <c r="AI256">
         <f t="shared" si="162"/>
-        <v>0.52879702927487948</v>
+        <v>0.54932859324135341</v>
       </c>
       <c r="AJ256">
         <f t="shared" si="150"/>
@@ -28384,19 +28428,19 @@
       </c>
       <c r="AL256">
         <f t="shared" si="163"/>
-        <v>4.1298036080372741E-4</v>
+        <v>4.2901511936953545E-4</v>
       </c>
       <c r="AM256">
         <f t="shared" si="164"/>
-        <v>3.1769224820969987E-4</v>
+        <v>3.3002726212744962E-4</v>
       </c>
       <c r="AN256">
         <f t="shared" si="165"/>
-        <v>7.3067260901342728E-4</v>
+        <v>7.5904238149698507E-4</v>
       </c>
       <c r="AO256">
         <f t="shared" si="166"/>
-        <v>0.30688249578563942</v>
+        <v>0.31879780022873372</v>
       </c>
     </row>
     <row r="257" spans="5:41" x14ac:dyDescent="0.2">
@@ -28426,9 +28470,11 @@
         <f>Tables!CC78</f>
         <v>0.65</v>
       </c>
-      <c r="Q257">
-        <f>Tables!CC114</f>
-        <v>65</v>
+      <c r="P257" s="1">
+        <v>68</v>
+      </c>
+      <c r="Q257" s="1">
+        <v>68</v>
       </c>
       <c r="R257">
         <f>$R$231</f>
@@ -28479,15 +28525,15 @@
       </c>
       <c r="AE257">
         <f t="shared" si="158"/>
-        <v>1.3486207988995054</v>
+        <v>1.4168488294882187</v>
       </c>
       <c r="AF257">
         <f t="shared" si="159"/>
-        <v>1.3465522699157941</v>
+        <v>1.4146756516225614</v>
       </c>
       <c r="AG257">
         <f t="shared" si="161"/>
-        <v>0.17505179508905325</v>
+        <v>0.18390783471093297</v>
       </c>
       <c r="AH257">
         <f t="shared" si="148"/>
@@ -28495,7 +28541,7 @@
       </c>
       <c r="AI257">
         <f t="shared" si="162"/>
-        <v>0.50031570188753161</v>
+        <v>0.52917366475647365</v>
       </c>
       <c r="AJ257">
         <f t="shared" si="150"/>
@@ -28507,19 +28553,19 @@
       </c>
       <c r="AL257">
         <f t="shared" si="163"/>
-        <v>3.9073698913288962E-4</v>
+        <v>4.132745059075558E-4</v>
       </c>
       <c r="AM257">
         <f t="shared" si="164"/>
-        <v>3.005811518366914E-4</v>
+        <v>3.1791852439182455E-4</v>
       </c>
       <c r="AN257">
         <f t="shared" si="165"/>
-        <v>6.9131814096958107E-4</v>
+        <v>7.311930302993804E-4</v>
       </c>
       <c r="AO257">
         <f t="shared" si="166"/>
-        <v>0.21430862370057013</v>
+        <v>0.22666983939280794</v>
       </c>
     </row>
     <row r="258" spans="5:41" x14ac:dyDescent="0.2">
@@ -28549,9 +28595,11 @@
         <f>Tables!CC78</f>
         <v>0.65</v>
       </c>
-      <c r="Q258">
-        <f>Tables!CC114</f>
-        <v>65</v>
+      <c r="P258" s="1">
+        <v>67</v>
+      </c>
+      <c r="Q258" s="1">
+        <v>67</v>
       </c>
       <c r="R258">
         <f>$R$231</f>
@@ -28602,15 +28650,15 @@
       </c>
       <c r="AE258">
         <f t="shared" si="158"/>
-        <v>1.3486207988995054</v>
+        <v>1.3940034864345587</v>
       </c>
       <c r="AF258">
         <f t="shared" si="159"/>
-        <v>1.3465522699157941</v>
+        <v>1.3918653490000499</v>
       </c>
       <c r="AG258">
         <f t="shared" si="161"/>
-        <v>0.17505179508905325</v>
+        <v>0.18094249537000648</v>
       </c>
       <c r="AH258">
         <f t="shared" si="148"/>
@@ -28618,7 +28666,7 @@
       </c>
       <c r="AI258">
         <f t="shared" si="162"/>
-        <v>0.50031570188753161</v>
+        <v>0.51947288308870676</v>
       </c>
       <c r="AJ258">
         <f t="shared" si="150"/>
@@ -28630,19 +28678,19 @@
       </c>
       <c r="AL258">
         <f t="shared" si="163"/>
-        <v>3.9073698913288962E-4</v>
+        <v>4.0569838105918791E-4</v>
       </c>
       <c r="AM258">
         <f t="shared" si="164"/>
-        <v>3.005811518366914E-4</v>
+        <v>3.1209045999885634E-4</v>
       </c>
       <c r="AN258">
         <f t="shared" si="165"/>
-        <v>6.9131814096958107E-4</v>
+        <v>7.1778884105804419E-4</v>
       </c>
       <c r="AO258">
         <f t="shared" si="166"/>
-        <v>0.5184886057271858</v>
+        <v>0.53834163079353314</v>
       </c>
     </row>
     <row r="259" spans="5:41" x14ac:dyDescent="0.2">

</xml_diff>